<commit_message>
commit de dois dias, sorry
</commit_message>
<xml_diff>
--- a/DOCS/modelo_dicionario_de_dados.xlsx
+++ b/DOCS/modelo_dicionario_de_dados.xlsx
@@ -415,7 +415,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -480,11 +480,6 @@
       <name val="Consolas"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Consolas"/>
-      <family val="0"/>
     </font>
     <font>
       <b val="true"/>
@@ -612,7 +607,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="58">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -657,12 +652,8 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -681,10 +672,6 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -701,7 +688,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -721,7 +708,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -741,7 +728,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -761,7 +748,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -781,7 +768,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -817,7 +804,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -837,24 +824,8 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -865,7 +836,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1248,7 +1219,7 @@
       <c r="I11" s="10"/>
     </row>
     <row r="12" s="11" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -1322,1164 +1293,1164 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" s="17" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="16"/>
-    </row>
-    <row r="16" s="22" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+    <row r="15" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="15"/>
+    </row>
+    <row r="16" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20" t="s">
+      <c r="C16" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G16" s="19" t="s">
+      <c r="F16" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="18"/>
-      <c r="I16" s="21" t="s">
+      <c r="H16" s="16"/>
+      <c r="I16" s="19" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" s="22" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="18" t="s">
+    <row r="17" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20" t="s">
+      <c r="D17" s="18"/>
+      <c r="E17" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="F17" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="19" t="s">
+      <c r="F17" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="H17" s="18"/>
-      <c r="I17" s="21"/>
-    </row>
-    <row r="18" s="22" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="18" t="s">
+      <c r="H17" s="16"/>
+      <c r="I17" s="19"/>
+    </row>
+    <row r="18" s="20" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20" t="s">
+      <c r="C18" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="F18" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="19" t="n">
+      <c r="F18" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="18"/>
-      <c r="I18" s="21" t="s">
+      <c r="H18" s="16"/>
+      <c r="I18" s="19" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" s="17" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="16"/>
-    </row>
-    <row r="20" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="s">
+    <row r="19" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="15"/>
+    </row>
+    <row r="20" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25" t="s">
+      <c r="C20" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="F20" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="24" t="s">
+      <c r="F20" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="H20" s="23"/>
-      <c r="I20" s="26" t="s">
+      <c r="H20" s="21"/>
+      <c r="I20" s="24" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="21" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="23" t="s">
+    <row r="21" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25" t="s">
+      <c r="D21" s="23"/>
+      <c r="E21" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G21" s="24"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="26"/>
-    </row>
-    <row r="22" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="23" t="s">
+      <c r="F21" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="22"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="24"/>
+    </row>
+    <row r="22" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25" t="s">
+      <c r="D22" s="23"/>
+      <c r="E22" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="24"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="26"/>
-    </row>
-    <row r="23" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="23" t="s">
+      <c r="F22" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="22"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="24"/>
+    </row>
+    <row r="23" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25" t="s">
+      <c r="D23" s="23"/>
+      <c r="E23" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="24"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="26"/>
-    </row>
-    <row r="24" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="23" t="s">
+      <c r="F23" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="22"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="24"/>
+    </row>
+    <row r="24" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="B24" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="C24" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25" t="s">
+      <c r="C24" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="24" t="n">
+      <c r="F24" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="23"/>
-      <c r="I24" s="26" t="s">
+      <c r="H24" s="21"/>
+      <c r="I24" s="24" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="25" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="23" t="s">
+    <row r="25" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25" t="s">
+      <c r="D25" s="23"/>
+      <c r="E25" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="24"/>
-      <c r="H25" s="23"/>
-      <c r="I25" s="26"/>
-    </row>
-    <row r="26" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="23" t="s">
+      <c r="F25" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="22"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="24"/>
+    </row>
+    <row r="26" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25" t="s">
+      <c r="D26" s="23"/>
+      <c r="E26" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G26" s="24"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="26"/>
-    </row>
-    <row r="27" s="27" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
+      <c r="F26" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="22"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="24"/>
+    </row>
+    <row r="27" s="25" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25" t="s">
+      <c r="D27" s="23"/>
+      <c r="E27" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="F27" s="25" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="24"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="26"/>
-    </row>
-    <row r="28" s="17" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="16"/>
-    </row>
-    <row r="29" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
+      <c r="F27" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="22"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="24"/>
+    </row>
+    <row r="28" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="15"/>
+    </row>
+    <row r="29" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B29" s="28" t="s">
+      <c r="B29" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C29" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30" t="s">
+      <c r="C29" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="F29" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" s="29" t="s">
+      <c r="F29" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="H29" s="28"/>
-      <c r="I29" s="31" t="s">
+      <c r="H29" s="26"/>
+      <c r="I29" s="29" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="30" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+    <row r="30" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="B30" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="C30" s="29" t="s">
+      <c r="C30" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30" t="s">
+      <c r="D30" s="28"/>
+      <c r="E30" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="F30" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G30" s="29"/>
-      <c r="H30" s="28"/>
-      <c r="I30" s="31"/>
-    </row>
-    <row r="31" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="F30" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G30" s="27"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="29"/>
+    </row>
+    <row r="31" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="28" t="s">
+      <c r="B31" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="C31" s="29" t="s">
+      <c r="C31" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G31" s="29"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="31"/>
-    </row>
-    <row r="32" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G31" s="27"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="29"/>
+    </row>
+    <row r="32" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="28" t="s">
+      <c r="B32" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C32" s="29" t="s">
+      <c r="C32" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30" t="s">
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="G32" s="29"/>
-      <c r="H32" s="28"/>
-      <c r="I32" s="31"/>
-    </row>
-    <row r="33" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28" t="s">
+      <c r="G32" s="27"/>
+      <c r="H32" s="26"/>
+      <c r="I32" s="29"/>
+    </row>
+    <row r="33" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B33" s="28" t="s">
+      <c r="B33" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30" t="s">
+      <c r="C33" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="F33" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G33" s="29"/>
-      <c r="H33" s="28"/>
-      <c r="I33" s="31"/>
-    </row>
-    <row r="34" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
+      <c r="F33" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G33" s="27"/>
+      <c r="H33" s="26"/>
+      <c r="I33" s="29"/>
+    </row>
+    <row r="34" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="28" t="s">
+      <c r="B34" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="C34" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D34" s="30"/>
-      <c r="E34" s="30" t="s">
+      <c r="C34" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="F34" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G34" s="29"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="31"/>
-    </row>
-    <row r="35" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="28" t="s">
+      <c r="F34" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G34" s="27"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="29"/>
+    </row>
+    <row r="35" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B35" s="28" t="s">
+      <c r="B35" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D35" s="30"/>
-      <c r="E35" s="30" t="s">
+      <c r="C35" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="F35" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G35" s="29"/>
-      <c r="H35" s="28"/>
-      <c r="I35" s="31"/>
-    </row>
-    <row r="36" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="28" t="s">
+      <c r="F35" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G35" s="27"/>
+      <c r="H35" s="26"/>
+      <c r="I35" s="29"/>
+    </row>
+    <row r="36" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="28" t="s">
+      <c r="B36" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D36" s="30"/>
-      <c r="E36" s="30" t="s">
+      <c r="C36" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28" t="s">
         <v>28</v>
       </c>
-      <c r="F36" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G36" s="29"/>
-      <c r="H36" s="28"/>
-      <c r="I36" s="31"/>
-    </row>
-    <row r="37" s="32" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="28" t="s">
+      <c r="F36" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="27"/>
+      <c r="H36" s="26"/>
+      <c r="I36" s="29"/>
+    </row>
+    <row r="37" s="30" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B37" s="28" t="s">
+      <c r="B37" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C37" s="29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D37" s="30"/>
-      <c r="E37" s="30" t="s">
+      <c r="C37" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="F37" s="30" t="s">
-        <v>21</v>
-      </c>
-      <c r="G37" s="29"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="31"/>
-    </row>
-    <row r="38" s="17" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13"/>
-      <c r="B38" s="13"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="16"/>
-    </row>
-    <row r="39" s="37" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="33" t="s">
+      <c r="F37" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="27"/>
+      <c r="H37" s="26"/>
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="13"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="15"/>
+    </row>
+    <row r="39" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="B39" s="33" t="s">
+      <c r="B39" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C39" s="34" t="s">
-        <v>19</v>
-      </c>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35" t="s">
+      <c r="C39" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="G39" s="34" t="s">
+      <c r="F39" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="H39" s="33"/>
-      <c r="I39" s="36" t="s">
+      <c r="H39" s="31"/>
+      <c r="I39" s="34" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="40" s="37" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="33" t="s">
+    <row r="40" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="B40" s="33" t="s">
+      <c r="B40" s="31" t="s">
         <v>58</v>
       </c>
-      <c r="C40" s="34" t="s">
+      <c r="C40" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35" t="s">
+      <c r="D40" s="33"/>
+      <c r="E40" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="F40" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="G40" s="34"/>
-      <c r="H40" s="33"/>
-      <c r="I40" s="36"/>
-    </row>
-    <row r="41" s="37" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="33" t="s">
+      <c r="F40" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="32"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="34"/>
+    </row>
+    <row r="41" s="35" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="33" t="s">
+      <c r="B41" s="31" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="34" t="s">
+      <c r="C41" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="D41" s="35"/>
-      <c r="E41" s="35" t="s">
+      <c r="D41" s="33"/>
+      <c r="E41" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="F41" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="G41" s="34" t="s">
+      <c r="F41" s="33" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="H41" s="33"/>
-      <c r="I41" s="36"/>
-    </row>
-    <row r="42" s="17" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13"/>
-      <c r="B42" s="13"/>
-      <c r="C42" s="14"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="13"/>
-      <c r="I42" s="16"/>
-    </row>
-    <row r="43" s="42" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="38" t="s">
+      <c r="H41" s="31"/>
+      <c r="I41" s="34"/>
+    </row>
+    <row r="42" s="1" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="15"/>
+    </row>
+    <row r="43" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B43" s="38" t="s">
+      <c r="B43" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C43" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D43" s="40"/>
-      <c r="E43" s="40" t="s">
+      <c r="C43" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="F43" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G43" s="39"/>
-      <c r="H43" s="38"/>
-      <c r="I43" s="41" t="s">
+      <c r="F43" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G43" s="37"/>
+      <c r="H43" s="36"/>
+      <c r="I43" s="39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="44" s="42" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="38" t="s">
+    <row r="44" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B44" s="38" t="s">
+      <c r="B44" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="C44" s="39" t="s">
+      <c r="C44" s="37" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="40"/>
-      <c r="E44" s="40" t="s">
+      <c r="D44" s="38"/>
+      <c r="E44" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="F44" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G44" s="39"/>
-      <c r="H44" s="38"/>
-      <c r="I44" s="41" t="s">
+      <c r="F44" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="37"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="45" s="42" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="38" t="s">
+    <row r="45" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="38" t="s">
+      <c r="B45" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="C45" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D45" s="40"/>
-      <c r="E45" s="40" t="s">
+      <c r="C45" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="F45" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G45" s="39"/>
-      <c r="H45" s="38"/>
-      <c r="I45" s="41" t="s">
+      <c r="F45" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="37"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="39" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="46" s="42" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="38" t="s">
+    <row r="46" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="38" t="s">
+      <c r="B46" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D46" s="40"/>
-      <c r="E46" s="40" t="s">
+      <c r="C46" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="F46" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G46" s="39"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="41"/>
-    </row>
-    <row r="47" s="42" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="38" t="s">
+      <c r="F46" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G46" s="37"/>
+      <c r="H46" s="36"/>
+      <c r="I46" s="39"/>
+    </row>
+    <row r="47" s="40" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="B47" s="38" t="s">
+      <c r="B47" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="39" t="s">
-        <v>19</v>
-      </c>
-      <c r="D47" s="40"/>
-      <c r="E47" s="40" t="s">
+      <c r="C47" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="F47" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="G47" s="39"/>
-      <c r="H47" s="38"/>
-      <c r="I47" s="41"/>
+      <c r="F47" s="38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G47" s="37"/>
+      <c r="H47" s="36"/>
+      <c r="I47" s="39"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="43"/>
-      <c r="B48" s="43"/>
-      <c r="C48" s="44"/>
-      <c r="D48" s="45"/>
-      <c r="E48" s="45"/>
-      <c r="F48" s="45"/>
-      <c r="G48" s="44"/>
-      <c r="H48" s="43"/>
-      <c r="I48" s="46"/>
-    </row>
-    <row r="49" s="51" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47" t="s">
+      <c r="A48" s="41"/>
+      <c r="B48" s="41"/>
+      <c r="C48" s="42"/>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="42"/>
+      <c r="H48" s="41"/>
+      <c r="I48" s="44"/>
+    </row>
+    <row r="49" s="49" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B49" s="47" t="s">
+      <c r="B49" s="45" t="s">
         <v>18</v>
       </c>
-      <c r="C49" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="D49" s="49"/>
-      <c r="E49" s="49" t="s">
+      <c r="C49" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="47"/>
+      <c r="E49" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="F49" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G49" s="48"/>
-      <c r="H49" s="47"/>
-      <c r="I49" s="50" t="s">
+      <c r="F49" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G49" s="46"/>
+      <c r="H49" s="45"/>
+      <c r="I49" s="48" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="50" s="51" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="47" t="s">
+    <row r="50" s="49" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B50" s="47" t="s">
+      <c r="B50" s="45" t="s">
         <v>62</v>
       </c>
-      <c r="C50" s="48" t="s">
+      <c r="C50" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="D50" s="49"/>
-      <c r="E50" s="49" t="s">
+      <c r="D50" s="47"/>
+      <c r="E50" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="F50" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G50" s="48"/>
-      <c r="H50" s="47"/>
-      <c r="I50" s="50" t="s">
+      <c r="F50" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="46"/>
+      <c r="H50" s="45"/>
+      <c r="I50" s="48" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" s="51" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="47" t="s">
+    <row r="51" s="49" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B51" s="47" t="s">
+      <c r="B51" s="45" t="s">
         <v>31</v>
       </c>
-      <c r="C51" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="D51" s="49"/>
-      <c r="E51" s="49" t="s">
+      <c r="C51" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="D51" s="47"/>
+      <c r="E51" s="47" t="s">
         <v>26</v>
       </c>
-      <c r="F51" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G51" s="48"/>
-      <c r="H51" s="47"/>
-      <c r="I51" s="50" t="s">
+      <c r="F51" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" s="46"/>
+      <c r="H51" s="45"/>
+      <c r="I51" s="48" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" s="51" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="47" t="s">
+    <row r="52" s="49" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B52" s="47" t="s">
+      <c r="B52" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="C52" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="D52" s="49"/>
-      <c r="E52" s="49" t="s">
+      <c r="C52" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="F52" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G52" s="48"/>
-      <c r="H52" s="47"/>
-      <c r="I52" s="50"/>
-    </row>
-    <row r="53" s="51" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="47" t="s">
+      <c r="F52" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="46"/>
+      <c r="H52" s="45"/>
+      <c r="I52" s="48"/>
+    </row>
+    <row r="53" s="49" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="45" t="s">
         <v>61</v>
       </c>
-      <c r="B53" s="47" t="s">
+      <c r="B53" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="C53" s="48" t="s">
-        <v>19</v>
-      </c>
-      <c r="D53" s="49"/>
-      <c r="E53" s="49" t="s">
+      <c r="C53" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" s="47"/>
+      <c r="E53" s="47" t="s">
         <v>28</v>
       </c>
-      <c r="F53" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="G53" s="48"/>
-      <c r="H53" s="47"/>
-      <c r="I53" s="50"/>
+      <c r="F53" s="47" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="46"/>
+      <c r="H53" s="45"/>
+      <c r="I53" s="48"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="43"/>
-      <c r="B54" s="43"/>
-      <c r="C54" s="44"/>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
-      <c r="F54" s="45"/>
-      <c r="G54" s="44"/>
-      <c r="H54" s="43"/>
-      <c r="I54" s="46"/>
-    </row>
-    <row r="55" s="56" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="52" t="s">
+      <c r="A54" s="41"/>
+      <c r="B54" s="41"/>
+      <c r="C54" s="42"/>
+      <c r="D54" s="43"/>
+      <c r="E54" s="43"/>
+      <c r="F54" s="43"/>
+      <c r="G54" s="42"/>
+      <c r="H54" s="41"/>
+      <c r="I54" s="44"/>
+    </row>
+    <row r="55" s="54" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B55" s="52" t="s">
+      <c r="B55" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C55" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D55" s="54"/>
-      <c r="E55" s="54" t="s">
+      <c r="C55" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D55" s="52"/>
+      <c r="E55" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="F55" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="G55" s="53"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="55" t="s">
+      <c r="F55" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="51"/>
+      <c r="H55" s="50"/>
+      <c r="I55" s="53" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" s="56" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="52" t="s">
+    <row r="56" s="54" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B56" s="52" t="s">
+      <c r="B56" s="50" t="s">
         <v>64</v>
       </c>
-      <c r="C56" s="53" t="s">
+      <c r="C56" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="D56" s="54"/>
-      <c r="E56" s="54" t="s">
+      <c r="D56" s="52"/>
+      <c r="E56" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="F56" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="G56" s="53"/>
-      <c r="H56" s="52"/>
-      <c r="I56" s="55" t="s">
+      <c r="F56" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G56" s="51"/>
+      <c r="H56" s="50"/>
+      <c r="I56" s="53" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" s="56" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="52" t="s">
+    <row r="57" s="54" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B57" s="52" t="s">
+      <c r="B57" s="50" t="s">
         <v>31</v>
       </c>
-      <c r="C57" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D57" s="54"/>
-      <c r="E57" s="54" t="s">
+      <c r="C57" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D57" s="52"/>
+      <c r="E57" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="F57" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="G57" s="53"/>
-      <c r="H57" s="52"/>
-      <c r="I57" s="55" t="s">
+      <c r="F57" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G57" s="51"/>
+      <c r="H57" s="50"/>
+      <c r="I57" s="53" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" s="56" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="52" t="s">
+    <row r="58" s="54" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B58" s="52" t="s">
+      <c r="B58" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C58" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D58" s="54"/>
-      <c r="E58" s="54" t="s">
+      <c r="C58" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D58" s="52"/>
+      <c r="E58" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="F58" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="G58" s="53"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="55"/>
-    </row>
-    <row r="59" s="56" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="52" t="s">
+      <c r="F58" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G58" s="51"/>
+      <c r="H58" s="50"/>
+      <c r="I58" s="53"/>
+    </row>
+    <row r="59" s="54" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="50" t="s">
         <v>63</v>
       </c>
-      <c r="B59" s="52" t="s">
+      <c r="B59" s="50" t="s">
         <v>46</v>
       </c>
-      <c r="C59" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D59" s="54"/>
-      <c r="E59" s="54" t="s">
+      <c r="C59" s="51" t="s">
+        <v>19</v>
+      </c>
+      <c r="D59" s="52"/>
+      <c r="E59" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="F59" s="54" t="s">
-        <v>21</v>
-      </c>
-      <c r="G59" s="53"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="55"/>
+      <c r="F59" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="G59" s="51"/>
+      <c r="H59" s="50"/>
+      <c r="I59" s="53"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="43"/>
-      <c r="B60" s="43"/>
-      <c r="C60" s="44"/>
-      <c r="D60" s="45"/>
-      <c r="E60" s="45"/>
-      <c r="F60" s="45"/>
-      <c r="G60" s="44"/>
-      <c r="H60" s="43"/>
-      <c r="I60" s="46"/>
+      <c r="A60" s="41"/>
+      <c r="B60" s="41"/>
+      <c r="C60" s="42"/>
+      <c r="D60" s="43"/>
+      <c r="E60" s="43"/>
+      <c r="F60" s="43"/>
+      <c r="G60" s="42"/>
+      <c r="H60" s="41"/>
+      <c r="I60" s="44"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A61" s="57"/>
-      <c r="B61" s="57"/>
-      <c r="C61" s="58"/>
-      <c r="D61" s="59"/>
-      <c r="E61" s="59"/>
-      <c r="F61" s="59"/>
-      <c r="G61" s="58"/>
-      <c r="H61" s="57"/>
-      <c r="I61" s="60"/>
+      <c r="A61" s="12"/>
+      <c r="B61" s="12"/>
+      <c r="C61" s="13"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="14"/>
+      <c r="F61" s="14"/>
+      <c r="G61" s="13"/>
+      <c r="H61" s="12"/>
+      <c r="I61" s="15"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="43"/>
-      <c r="B62" s="43"/>
-      <c r="C62" s="44"/>
-      <c r="D62" s="45"/>
-      <c r="E62" s="45"/>
-      <c r="F62" s="45"/>
-      <c r="G62" s="44"/>
-      <c r="H62" s="43"/>
-      <c r="I62" s="46"/>
+      <c r="A62" s="41"/>
+      <c r="B62" s="41"/>
+      <c r="C62" s="42"/>
+      <c r="D62" s="43"/>
+      <c r="E62" s="43"/>
+      <c r="F62" s="43"/>
+      <c r="G62" s="42"/>
+      <c r="H62" s="41"/>
+      <c r="I62" s="44"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="57"/>
-      <c r="B63" s="57"/>
-      <c r="C63" s="58"/>
-      <c r="D63" s="59"/>
-      <c r="E63" s="59"/>
-      <c r="F63" s="59"/>
-      <c r="G63" s="58"/>
-      <c r="H63" s="57"/>
-      <c r="I63" s="60"/>
+      <c r="A63" s="12"/>
+      <c r="B63" s="12"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="14"/>
+      <c r="F63" s="14"/>
+      <c r="G63" s="13"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="43"/>
-      <c r="B64" s="43"/>
-      <c r="C64" s="44"/>
-      <c r="D64" s="45"/>
-      <c r="E64" s="45"/>
-      <c r="F64" s="45"/>
-      <c r="G64" s="44"/>
-      <c r="H64" s="43"/>
-      <c r="I64" s="46"/>
+      <c r="A64" s="41"/>
+      <c r="B64" s="41"/>
+      <c r="C64" s="42"/>
+      <c r="D64" s="43"/>
+      <c r="E64" s="43"/>
+      <c r="F64" s="43"/>
+      <c r="G64" s="42"/>
+      <c r="H64" s="41"/>
+      <c r="I64" s="44"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="57"/>
-      <c r="B65" s="57"/>
-      <c r="C65" s="58"/>
-      <c r="D65" s="59"/>
-      <c r="E65" s="59"/>
-      <c r="F65" s="59"/>
-      <c r="G65" s="58"/>
-      <c r="H65" s="57"/>
-      <c r="I65" s="60"/>
+      <c r="A65" s="12"/>
+      <c r="B65" s="12"/>
+      <c r="C65" s="13"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="14"/>
+      <c r="F65" s="14"/>
+      <c r="G65" s="13"/>
+      <c r="H65" s="12"/>
+      <c r="I65" s="15"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="43"/>
-      <c r="B66" s="43"/>
-      <c r="C66" s="44"/>
-      <c r="D66" s="45"/>
-      <c r="E66" s="45"/>
-      <c r="F66" s="45"/>
-      <c r="G66" s="44"/>
-      <c r="H66" s="43"/>
-      <c r="I66" s="46"/>
+      <c r="A66" s="41"/>
+      <c r="B66" s="41"/>
+      <c r="C66" s="42"/>
+      <c r="D66" s="43"/>
+      <c r="E66" s="43"/>
+      <c r="F66" s="43"/>
+      <c r="G66" s="42"/>
+      <c r="H66" s="41"/>
+      <c r="I66" s="44"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="57"/>
-      <c r="B67" s="57"/>
-      <c r="C67" s="58"/>
-      <c r="D67" s="59"/>
-      <c r="E67" s="59"/>
-      <c r="F67" s="59"/>
-      <c r="G67" s="58"/>
-      <c r="H67" s="57"/>
-      <c r="I67" s="60"/>
+      <c r="A67" s="12"/>
+      <c r="B67" s="12"/>
+      <c r="C67" s="13"/>
+      <c r="D67" s="14"/>
+      <c r="E67" s="14"/>
+      <c r="F67" s="14"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="12"/>
+      <c r="I67" s="15"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="43"/>
-      <c r="B68" s="43"/>
-      <c r="C68" s="44"/>
-      <c r="D68" s="45"/>
-      <c r="E68" s="45"/>
-      <c r="F68" s="45"/>
-      <c r="G68" s="44"/>
-      <c r="H68" s="43"/>
-      <c r="I68" s="46"/>
+      <c r="A68" s="41"/>
+      <c r="B68" s="41"/>
+      <c r="C68" s="42"/>
+      <c r="D68" s="43"/>
+      <c r="E68" s="43"/>
+      <c r="F68" s="43"/>
+      <c r="G68" s="42"/>
+      <c r="H68" s="41"/>
+      <c r="I68" s="44"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="57"/>
-      <c r="B69" s="57"/>
-      <c r="C69" s="58"/>
-      <c r="D69" s="59"/>
-      <c r="E69" s="59"/>
-      <c r="F69" s="59"/>
-      <c r="G69" s="58"/>
-      <c r="H69" s="57"/>
-      <c r="I69" s="60"/>
+      <c r="A69" s="12"/>
+      <c r="B69" s="12"/>
+      <c r="C69" s="13"/>
+      <c r="D69" s="14"/>
+      <c r="E69" s="14"/>
+      <c r="F69" s="14"/>
+      <c r="G69" s="13"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="15"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="43"/>
-      <c r="B70" s="43"/>
-      <c r="C70" s="44"/>
-      <c r="D70" s="45"/>
-      <c r="E70" s="45"/>
-      <c r="F70" s="45"/>
-      <c r="G70" s="44"/>
-      <c r="H70" s="43"/>
-      <c r="I70" s="46"/>
+      <c r="A70" s="41"/>
+      <c r="B70" s="41"/>
+      <c r="C70" s="42"/>
+      <c r="D70" s="43"/>
+      <c r="E70" s="43"/>
+      <c r="F70" s="43"/>
+      <c r="G70" s="42"/>
+      <c r="H70" s="41"/>
+      <c r="I70" s="44"/>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="57"/>
-      <c r="B71" s="57"/>
-      <c r="C71" s="58"/>
-      <c r="D71" s="59"/>
-      <c r="E71" s="59"/>
-      <c r="F71" s="59"/>
-      <c r="G71" s="58"/>
-      <c r="H71" s="57"/>
-      <c r="I71" s="60"/>
+      <c r="A71" s="12"/>
+      <c r="B71" s="12"/>
+      <c r="C71" s="13"/>
+      <c r="D71" s="14"/>
+      <c r="E71" s="14"/>
+      <c r="F71" s="14"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="12"/>
+      <c r="I71" s="15"/>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="43"/>
-      <c r="B72" s="43"/>
-      <c r="C72" s="44"/>
-      <c r="D72" s="45"/>
-      <c r="E72" s="45"/>
-      <c r="F72" s="45"/>
-      <c r="G72" s="44"/>
-      <c r="H72" s="43"/>
-      <c r="I72" s="46"/>
+      <c r="A72" s="41"/>
+      <c r="B72" s="41"/>
+      <c r="C72" s="42"/>
+      <c r="D72" s="43"/>
+      <c r="E72" s="43"/>
+      <c r="F72" s="43"/>
+      <c r="G72" s="42"/>
+      <c r="H72" s="41"/>
+      <c r="I72" s="44"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="57"/>
-      <c r="B73" s="57"/>
-      <c r="C73" s="58"/>
-      <c r="D73" s="59"/>
-      <c r="E73" s="59"/>
-      <c r="F73" s="59"/>
-      <c r="G73" s="58"/>
-      <c r="H73" s="57"/>
-      <c r="I73" s="60"/>
+      <c r="A73" s="12"/>
+      <c r="B73" s="12"/>
+      <c r="C73" s="13"/>
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="14"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="12"/>
+      <c r="I73" s="15"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="43"/>
-      <c r="B74" s="43"/>
-      <c r="C74" s="44"/>
-      <c r="D74" s="45"/>
-      <c r="E74" s="45"/>
-      <c r="F74" s="45"/>
-      <c r="G74" s="44"/>
-      <c r="H74" s="43"/>
-      <c r="I74" s="46"/>
+      <c r="A74" s="41"/>
+      <c r="B74" s="41"/>
+      <c r="C74" s="42"/>
+      <c r="D74" s="43"/>
+      <c r="E74" s="43"/>
+      <c r="F74" s="43"/>
+      <c r="G74" s="42"/>
+      <c r="H74" s="41"/>
+      <c r="I74" s="44"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="57"/>
-      <c r="B75" s="57"/>
-      <c r="C75" s="58"/>
-      <c r="D75" s="59"/>
-      <c r="E75" s="59"/>
-      <c r="F75" s="59"/>
-      <c r="G75" s="58"/>
-      <c r="H75" s="57"/>
-      <c r="I75" s="60"/>
+      <c r="A75" s="12"/>
+      <c r="B75" s="12"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="14"/>
+      <c r="G75" s="13"/>
+      <c r="H75" s="12"/>
+      <c r="I75" s="15"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="43"/>
-      <c r="B76" s="43"/>
-      <c r="C76" s="44"/>
-      <c r="D76" s="45"/>
-      <c r="E76" s="45"/>
-      <c r="F76" s="45"/>
-      <c r="G76" s="44"/>
-      <c r="H76" s="43"/>
-      <c r="I76" s="46"/>
+      <c r="A76" s="41"/>
+      <c r="B76" s="41"/>
+      <c r="C76" s="42"/>
+      <c r="D76" s="43"/>
+      <c r="E76" s="43"/>
+      <c r="F76" s="43"/>
+      <c r="G76" s="42"/>
+      <c r="H76" s="41"/>
+      <c r="I76" s="44"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="57"/>
-      <c r="B77" s="57"/>
-      <c r="C77" s="58"/>
-      <c r="D77" s="59"/>
-      <c r="E77" s="59"/>
-      <c r="F77" s="59"/>
-      <c r="G77" s="58"/>
-      <c r="H77" s="57"/>
-      <c r="I77" s="60"/>
+      <c r="A77" s="12"/>
+      <c r="B77" s="12"/>
+      <c r="C77" s="13"/>
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="14"/>
+      <c r="G77" s="13"/>
+      <c r="H77" s="12"/>
+      <c r="I77" s="15"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="43"/>
-      <c r="B78" s="43"/>
-      <c r="C78" s="44"/>
-      <c r="D78" s="45"/>
-      <c r="E78" s="45"/>
-      <c r="F78" s="45"/>
-      <c r="G78" s="44"/>
-      <c r="H78" s="43"/>
-      <c r="I78" s="46"/>
+      <c r="A78" s="41"/>
+      <c r="B78" s="41"/>
+      <c r="C78" s="42"/>
+      <c r="D78" s="43"/>
+      <c r="E78" s="43"/>
+      <c r="F78" s="43"/>
+      <c r="G78" s="42"/>
+      <c r="H78" s="41"/>
+      <c r="I78" s="44"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="57"/>
-      <c r="B79" s="57"/>
-      <c r="C79" s="58"/>
-      <c r="D79" s="59"/>
-      <c r="E79" s="59"/>
-      <c r="F79" s="59"/>
-      <c r="G79" s="58"/>
-      <c r="H79" s="57"/>
-      <c r="I79" s="60"/>
+      <c r="A79" s="12"/>
+      <c r="B79" s="12"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="14"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="14"/>
+      <c r="G79" s="13"/>
+      <c r="H79" s="12"/>
+      <c r="I79" s="15"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="43"/>
-      <c r="B80" s="43"/>
-      <c r="C80" s="44"/>
-      <c r="D80" s="45"/>
-      <c r="E80" s="45"/>
-      <c r="F80" s="45"/>
-      <c r="G80" s="44"/>
-      <c r="H80" s="43"/>
-      <c r="I80" s="46"/>
+      <c r="A80" s="41"/>
+      <c r="B80" s="41"/>
+      <c r="C80" s="42"/>
+      <c r="D80" s="43"/>
+      <c r="E80" s="43"/>
+      <c r="F80" s="43"/>
+      <c r="G80" s="42"/>
+      <c r="H80" s="41"/>
+      <c r="I80" s="44"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="57"/>
-      <c r="B81" s="57"/>
-      <c r="C81" s="58"/>
-      <c r="D81" s="59"/>
-      <c r="E81" s="59"/>
-      <c r="F81" s="59"/>
-      <c r="G81" s="58"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="60"/>
+      <c r="A81" s="12"/>
+      <c r="B81" s="12"/>
+      <c r="C81" s="13"/>
+      <c r="D81" s="14"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="14"/>
+      <c r="G81" s="13"/>
+      <c r="H81" s="12"/>
+      <c r="I81" s="15"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2535,79 +2506,79 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="61" t="s">
+      <c r="A4" s="55" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="56" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="61" t="s">
+      <c r="A5" s="55" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="56" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="61" t="s">
+      <c r="A6" s="55" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="56" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="61" t="s">
+      <c r="A7" s="55" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="56" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="61" t="s">
+      <c r="A8" s="55" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="56" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="61" t="s">
+      <c r="A9" s="55" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="62" t="s">
+      <c r="B9" s="56" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="55" t="s">
         <v>79</v>
       </c>
-      <c r="B10" s="62" t="s">
+      <c r="B10" s="56" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="55" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="62" t="s">
+      <c r="B11" s="56" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="61" t="s">
+      <c r="A12" s="55" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="56" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="63" t="s">
+      <c r="A14" s="57" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2641,245 +2612,245 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="57" t="s">
+      <c r="A17" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="59" t="s">
+      <c r="C17" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="59" t="s">
+      <c r="E17" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" s="58" t="s">
+      <c r="F17" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="H17" s="57" t="s">
+      <c r="H17" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="I17" s="60" t="s">
+      <c r="I17" s="15" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="43" t="s">
+      <c r="A18" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="B18" s="43" t="s">
+      <c r="B18" s="41" t="s">
         <v>95</v>
       </c>
-      <c r="C18" s="44" t="s">
+      <c r="C18" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="43" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="45" t="s">
+      <c r="E18" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="F18" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="44" t="s">
+      <c r="F18" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="H18" s="43" t="s">
+      <c r="H18" s="41" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="57" t="s">
+      <c r="A19" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="59" t="s">
+      <c r="D19" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E19" s="59" t="s">
+      <c r="E19" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F19" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="G19" s="58" t="s">
+      <c r="F19" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G19" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="H19" s="57" t="s">
+      <c r="H19" s="12" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="43" t="s">
+      <c r="A20" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="B20" s="43" t="s">
+      <c r="B20" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="44" t="s">
+      <c r="C20" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D20" s="43" t="s">
         <v>93</v>
       </c>
-      <c r="E20" s="45" t="s">
+      <c r="E20" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="F20" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G20" s="44" t="s">
+      <c r="F20" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="H20" s="43" t="s">
+      <c r="H20" s="41" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="57" t="s">
+      <c r="A21" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="D21" s="59" t="s">
+      <c r="D21" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="E21" s="59" t="s">
+      <c r="E21" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="59" t="s">
+      <c r="F21" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="58" t="s">
+      <c r="G21" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="H21" s="57" t="s">
+      <c r="H21" s="12" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="43" t="s">
+      <c r="A22" s="41" t="s">
         <v>89</v>
       </c>
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="41" t="s">
         <v>107</v>
       </c>
-      <c r="C22" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D22" s="45" t="s">
+      <c r="C22" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="43" t="s">
         <v>91</v>
       </c>
-      <c r="E22" s="45" t="s">
+      <c r="E22" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="F22" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G22" s="44" t="s">
+      <c r="F22" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="H22" s="43" t="s">
+      <c r="H22" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="I22" s="46" t="s">
+      <c r="I22" s="44" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="57" t="s">
+      <c r="A23" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="B23" s="57" t="s">
+      <c r="B23" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="C23" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" s="59" t="s">
+      <c r="C23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E23" s="59" t="s">
+      <c r="E23" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="G23" s="58" t="s">
+      <c r="F23" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G23" s="13" t="s">
         <v>92</v>
       </c>
-      <c r="H23" s="57" t="s">
+      <c r="H23" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="I23" s="60" t="s">
+      <c r="I23" s="15" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="41" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="44" t="s">
+      <c r="C24" s="42" t="s">
         <v>96</v>
       </c>
-      <c r="D24" s="45" t="s">
+      <c r="D24" s="43" t="s">
         <v>113</v>
       </c>
-      <c r="E24" s="45" t="s">
+      <c r="E24" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="F24" s="45" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="44" t="s">
+      <c r="F24" s="43" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="H24" s="43" t="s">
+      <c r="H24" s="41" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="57" t="s">
+      <c r="A25" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C25" s="58" t="s">
-        <v>19</v>
-      </c>
-      <c r="D25" s="59" t="s">
+      <c r="C25" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D25" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="E25" s="59" t="s">
+      <c r="E25" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="F25" s="59" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="58" t="s">
+      <c r="F25" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="H25" s="57" t="s">
+      <c r="H25" s="12" t="s">
         <v>118</v>
       </c>
     </row>

</xml_diff>